<commit_message>
remove ACC1 from experimental dataset for sclareol production.
</commit_message>
<xml_diff>
--- a/data/experiment_targets/detailed_collect/sclareol_exp_data.xlsx
+++ b/data/experiment_targets/detailed_collect/sclareol_exp_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\github\strainOptimizer\data\experiment_targets\detailed_collect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F10429-8343-4F5B-B081-6E347305C598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCE894F-CE92-4B9E-84AA-AD69A7982B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4140" yWindow="1050" windowWidth="16410" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28575" yWindow="5895" windowWidth="15930" windowHeight="18465" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="85">
   <si>
     <t>geneID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -160,10 +160,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ACC1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>PYC1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -201,10 +197,6 @@
   </si>
   <si>
     <t>YGL062W</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>YNR016C</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1363,7 +1355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="30.25" customWidth="1"/>
@@ -1389,27 +1381,27 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="M1" t="s">
+        <v>64</v>
+      </c>
+      <c r="N1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P1" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q1" t="s">
         <v>66</v>
-      </c>
-      <c r="N1" t="s">
-        <v>54</v>
-      </c>
-      <c r="O1" t="s">
-        <v>76</v>
-      </c>
-      <c r="P1" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -1421,16 +1413,16 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
         <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M2">
         <v>0.16</v>
@@ -1441,7 +1433,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -1456,10 +1448,10 @@
         <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M3">
         <v>2.4E-2</v>
@@ -1470,7 +1462,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -1485,10 +1477,10 @@
         <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="M4">
         <v>8.1999999999999993</v>
@@ -1499,7 +1491,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -1514,10 +1506,10 @@
         <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M5">
         <v>14.8</v>
@@ -1528,10 +1520,10 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -1543,10 +1535,10 @@
         <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M6">
         <v>4.8000000000000001E-2</v>
@@ -1572,10 +1564,10 @@
         <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="M7">
         <v>584</v>
@@ -1610,10 +1602,10 @@
         <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M8">
         <v>35</v>
@@ -1633,7 +1625,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
         <v>18</v>
@@ -1648,7 +1640,7 @@
         <v>16</v>
       </c>
       <c r="G9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -1665,10 +1657,10 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -1688,12 +1680,12 @@
         <v>22</v>
       </c>
       <c r="G11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
@@ -1708,7 +1700,7 @@
         <v>22</v>
       </c>
       <c r="G12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
@@ -1728,7 +1720,7 @@
         <v>22</v>
       </c>
       <c r="G13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
@@ -1748,12 +1740,12 @@
         <v>22</v>
       </c>
       <c r="G14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -1768,55 +1760,55 @@
         <v>22</v>
       </c>
       <c r="G15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="G16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
         <v>13</v>
@@ -1825,18 +1817,18 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
         <v>13</v>
@@ -1845,18 +1837,18 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C20" t="s">
         <v>13</v>
@@ -1865,18 +1857,18 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
         <v>13</v>
@@ -1885,38 +1877,38 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
         <v>13</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G22" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" t="s">
         <v>13</v>
@@ -1925,30 +1917,10 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G23" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" t="s">
-        <v>48</v>
-      </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="F24" t="s">
-        <v>50</v>
-      </c>
-      <c r="G24" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1965,55 +1937,56 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>